<commit_message>
update component values RX
</commit_message>
<xml_diff>
--- a/Receiver/Schematics/Rx_Component_Values.xlsx
+++ b/Receiver/Schematics/Rx_Component_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kburd\Projects\310_Projects\310-water-sensing\Receiver\Schematics\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmstr\Documents\GitHub\310-water-sensing\Receiver\Schematics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2095C2D7-3BB6-4292-A9F9-F8FB91C2A1A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3D17758-CA14-4B1B-8B3E-17C2BF0BC68B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{F40470B7-ED99-4AB5-B240-6294F62437B9}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{F40470B7-ED99-4AB5-B240-6294F62437B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="86">
   <si>
     <t>Component</t>
   </si>
@@ -246,6 +246,57 @@
   </si>
   <si>
     <t>100n</t>
+  </si>
+  <si>
+    <t>33k</t>
+  </si>
+  <si>
+    <t>47k</t>
+  </si>
+  <si>
+    <t>82k</t>
+  </si>
+  <si>
+    <t>56k</t>
+  </si>
+  <si>
+    <t>470n</t>
+  </si>
+  <si>
+    <t>220n</t>
+  </si>
+  <si>
+    <t>5.6k</t>
+  </si>
+  <si>
+    <t>3.3k</t>
+  </si>
+  <si>
+    <t>120p</t>
+  </si>
+  <si>
+    <t>2.2k</t>
+  </si>
+  <si>
+    <t>10k</t>
+  </si>
+  <si>
+    <t>180p</t>
+  </si>
+  <si>
+    <t>3.9k</t>
+  </si>
+  <si>
+    <t>100p</t>
+  </si>
+  <si>
+    <t>470k</t>
+  </si>
+  <si>
+    <t>4.7n</t>
+  </si>
+  <si>
+    <t>470p</t>
   </si>
 </sst>
 </file>
@@ -509,6 +560,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -535,15 +595,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -897,23 +948,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83595E41-0051-4B9D-8826-7E3F5EB5C3FC}">
   <dimension ref="A1:D63"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="22.88671875" customWidth="1"/>
+    <col min="1" max="1" width="22.86328125" customWidth="1"/>
     <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.19921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.53125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="57.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:4" ht="57.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="14"/>
-    </row>
-    <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="17"/>
+    </row>
+    <row r="2" spans="1:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A2" s="2" t="s">
         <v>61</v>
       </c>
@@ -927,600 +978,666 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
       <c r="D3" s="8"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="15" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A4" s="18" t="s">
         <v>53</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="12" t="s">
         <v>67</v>
       </c>
       <c r="D4" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="17"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A5" s="20"/>
       <c r="B5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="13" t="s">
         <v>68</v>
       </c>
       <c r="D5" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" s="1"/>
-      <c r="C6" s="23"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="15" t="s">
+      <c r="C6" s="14"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A7" s="18" t="s">
         <v>54</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="21"/>
+      <c r="C7" s="12" t="s">
+        <v>76</v>
+      </c>
       <c r="D7" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A8" s="19"/>
       <c r="B8" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="23"/>
+      <c r="C8" s="14">
+        <v>820</v>
+      </c>
       <c r="D8" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A9" s="19"/>
       <c r="B9" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="14" t="s">
         <v>64</v>
       </c>
       <c r="D9" s="7" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="16"/>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A10" s="19"/>
       <c r="B10" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="23" t="s">
+      <c r="C10" s="14" t="s">
         <v>64</v>
       </c>
       <c r="D10" s="7" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="17"/>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A11" s="20"/>
       <c r="B11" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="22"/>
+      <c r="C11" s="13" t="s">
+        <v>77</v>
+      </c>
       <c r="D11" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" s="1"/>
-      <c r="C12" s="23"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="15" t="s">
+      <c r="C12" s="14"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A13" s="18" t="s">
         <v>55</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="21"/>
+      <c r="C13" s="12" t="s">
+        <v>78</v>
+      </c>
       <c r="D13" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A14" s="19"/>
       <c r="B14" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="23"/>
+      <c r="C14" s="14">
+        <v>120</v>
+      </c>
       <c r="D14" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A15" s="19"/>
       <c r="B15" t="s">
         <v>10</v>
       </c>
-      <c r="C15" s="23"/>
+      <c r="C15" s="14" t="s">
+        <v>79</v>
+      </c>
       <c r="D15" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A16" s="19"/>
       <c r="B16" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="23"/>
+      <c r="C16" s="14" t="s">
+        <v>80</v>
+      </c>
       <c r="D16" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="17"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A17" s="20"/>
       <c r="B17" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="22"/>
+      <c r="C17" s="13" t="s">
+        <v>68</v>
+      </c>
       <c r="D17" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A18" s="1"/>
-      <c r="C18" s="23"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="15" t="s">
+      <c r="C18" s="14"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A19" s="18" t="s">
         <v>56</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="21"/>
+      <c r="C19" s="12"/>
       <c r="D19" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="16"/>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A20" s="19"/>
       <c r="B20" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="23"/>
+      <c r="C20" s="14">
+        <v>120</v>
+      </c>
       <c r="D20" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A21" s="19"/>
       <c r="B21" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="23" t="s">
+      <c r="C21" s="14" t="s">
         <v>64</v>
       </c>
       <c r="D21" s="7" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="17"/>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A22" s="20"/>
       <c r="B22" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C22" s="22"/>
+      <c r="C22" s="13" t="s">
+        <v>81</v>
+      </c>
       <c r="D22" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" s="1"/>
-      <c r="C23" s="23"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="18" t="s">
+      <c r="C23" s="14"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A24" s="21" t="s">
         <v>63</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C24" s="21" t="s">
+      <c r="C24" s="12" t="s">
         <v>64</v>
       </c>
       <c r="D24" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="19"/>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A25" s="22"/>
       <c r="B25" t="s">
         <v>20</v>
       </c>
-      <c r="C25" s="23" t="s">
-        <v>64</v>
+      <c r="C25" s="14" t="s">
+        <v>83</v>
       </c>
       <c r="D25" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="19"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A26" s="22"/>
       <c r="B26" t="s">
         <v>21</v>
       </c>
-      <c r="C26" s="23" t="s">
+      <c r="C26" s="14" t="s">
         <v>64</v>
       </c>
       <c r="D26" s="7" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="19"/>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A27" s="22"/>
       <c r="B27" t="s">
         <v>22</v>
       </c>
-      <c r="C27" s="23"/>
+      <c r="C27" s="14"/>
       <c r="D27" s="7" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="19"/>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A28" s="22"/>
       <c r="B28" t="s">
         <v>65</v>
       </c>
-      <c r="C28" s="23"/>
+      <c r="C28" s="14"/>
       <c r="D28" s="7" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="19"/>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A29" s="22"/>
       <c r="B29" t="s">
         <v>23</v>
       </c>
-      <c r="C29" s="23" t="s">
-        <v>64</v>
+      <c r="C29" s="14" t="s">
+        <v>82</v>
       </c>
       <c r="D29" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="19"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A30" s="22"/>
       <c r="B30" t="s">
         <v>50</v>
       </c>
-      <c r="C30" s="23"/>
+      <c r="C30" s="14" t="s">
+        <v>84</v>
+      </c>
       <c r="D30" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="20"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A31" s="23"/>
       <c r="B31" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C31" s="22"/>
+      <c r="C31" s="13"/>
       <c r="D31" s="6" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A32" s="1"/>
-      <c r="C32" s="23"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="15" t="s">
+      <c r="C32" s="14"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A33" s="18" t="s">
         <v>57</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C33" s="21"/>
+      <c r="C33" s="12" t="s">
+        <v>70</v>
+      </c>
       <c r="D33" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A34" s="19"/>
       <c r="B34" t="s">
         <v>27</v>
       </c>
-      <c r="C34" s="23"/>
+      <c r="C34" s="14" t="s">
+        <v>72</v>
+      </c>
       <c r="D34" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A35" s="19"/>
       <c r="B35" t="s">
         <v>28</v>
       </c>
-      <c r="C35" s="23"/>
+      <c r="C35" s="14" t="s">
+        <v>75</v>
+      </c>
       <c r="D35" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A36" s="19"/>
       <c r="B36" t="s">
         <v>29</v>
       </c>
-      <c r="C36" s="23"/>
+      <c r="C36" s="14" t="s">
+        <v>71</v>
+      </c>
       <c r="D36" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A37" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A37" s="19"/>
       <c r="B37" t="s">
         <v>30</v>
       </c>
-      <c r="C37" s="23"/>
+      <c r="C37" s="14" t="s">
+        <v>70</v>
+      </c>
       <c r="D37" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A38" s="19"/>
       <c r="B38" t="s">
         <v>66</v>
       </c>
-      <c r="C38" s="23" t="s">
+      <c r="C38" s="14" t="s">
         <v>64</v>
       </c>
       <c r="D38" s="7" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A39" s="16"/>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A39" s="19"/>
       <c r="B39" t="s">
         <v>31</v>
       </c>
-      <c r="C39" s="23"/>
+      <c r="C39" s="14" t="s">
+        <v>69</v>
+      </c>
       <c r="D39" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A40" s="19"/>
       <c r="B40" t="s">
         <v>32</v>
       </c>
-      <c r="C40" s="23"/>
+      <c r="C40" s="14" t="s">
+        <v>73</v>
+      </c>
       <c r="D40" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A41" s="19"/>
       <c r="B41" t="s">
         <v>33</v>
       </c>
-      <c r="C41" s="23"/>
+      <c r="C41" s="14" t="s">
+        <v>73</v>
+      </c>
       <c r="D41" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A42" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A42" s="19"/>
       <c r="B42" t="s">
         <v>34</v>
       </c>
-      <c r="C42" s="23"/>
+      <c r="C42" s="14" t="s">
+        <v>74</v>
+      </c>
       <c r="D42" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A43" s="17"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A43" s="20"/>
       <c r="B43" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C43" s="22"/>
+      <c r="C43" s="13" t="s">
+        <v>68</v>
+      </c>
       <c r="D43" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A44" s="1"/>
-      <c r="C44" s="23"/>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A45" s="15" t="s">
+      <c r="C44" s="14"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A45" s="18" t="s">
         <v>58</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C45" s="21"/>
+      <c r="C45" s="12"/>
       <c r="D45" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A46" s="16"/>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A46" s="19"/>
       <c r="B46" t="s">
         <v>37</v>
       </c>
-      <c r="C46" s="23"/>
+      <c r="C46" s="14"/>
       <c r="D46" s="7" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A47" s="16"/>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A47" s="19"/>
       <c r="B47" t="s">
         <v>38</v>
       </c>
-      <c r="C47" s="23"/>
+      <c r="C47" s="14"/>
       <c r="D47" s="7" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A48" s="16"/>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A48" s="19"/>
       <c r="B48" t="s">
         <v>39</v>
       </c>
-      <c r="C48" s="23"/>
+      <c r="C48" s="14"/>
       <c r="D48" s="7" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" s="17"/>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A49" s="20"/>
       <c r="B49" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C49" s="22"/>
+      <c r="C49" s="13"/>
       <c r="D49" s="6" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A50" s="1"/>
-      <c r="C50" s="23"/>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A51" s="15" t="s">
+      <c r="C50" s="14"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A51" s="18" t="s">
         <v>59</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C51" s="21"/>
+      <c r="C51" s="12" t="s">
+        <v>79</v>
+      </c>
       <c r="D51" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A52" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A52" s="19"/>
       <c r="B52" t="s">
         <v>42</v>
       </c>
-      <c r="C52" s="23"/>
+      <c r="C52" s="14">
+        <v>47</v>
+      </c>
       <c r="D52" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A53" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A53" s="19"/>
       <c r="B53" t="s">
         <v>43</v>
       </c>
-      <c r="C53" s="23"/>
+      <c r="C53" s="14" t="s">
+        <v>79</v>
+      </c>
       <c r="D53" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A54" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A54" s="19"/>
       <c r="B54" t="s">
         <v>44</v>
       </c>
-      <c r="C54" s="23"/>
+      <c r="C54" s="14" t="s">
+        <v>79</v>
+      </c>
       <c r="D54" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A55" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A55" s="19"/>
       <c r="B55" t="s">
         <v>45</v>
       </c>
-      <c r="C55" s="23"/>
+      <c r="C55" s="14" t="s">
+        <v>85</v>
+      </c>
       <c r="D55" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A56" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A56" s="19"/>
       <c r="B56" t="s">
         <v>46</v>
       </c>
-      <c r="C56" s="23"/>
+      <c r="C56" s="14" t="s">
+        <v>68</v>
+      </c>
       <c r="D56" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A57" s="17"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A57" s="20"/>
       <c r="B57" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C57" s="22"/>
+      <c r="C57" s="13" t="s">
+        <v>68</v>
+      </c>
       <c r="D57" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A58" s="1"/>
-      <c r="C58" s="23"/>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A59" s="15" t="s">
+      <c r="C58" s="14"/>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A59" s="18" t="s">
         <v>60</v>
       </c>
       <c r="B59" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C59" s="21"/>
+      <c r="C59" s="12" t="s">
+        <v>68</v>
+      </c>
       <c r="D59" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A60" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A60" s="19"/>
       <c r="B60" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C60" s="23"/>
+      <c r="C60" s="14" t="s">
+        <v>68</v>
+      </c>
       <c r="D60" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A61" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A61" s="19"/>
       <c r="B61" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C61" s="23"/>
+      <c r="C61" s="14" t="s">
+        <v>68</v>
+      </c>
       <c r="D61" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A62" s="16"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A62" s="19"/>
       <c r="B62" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C62" s="23"/>
+      <c r="C62" s="14" t="s">
+        <v>68</v>
+      </c>
       <c r="D62" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A63" s="17"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A63" s="20"/>
       <c r="B63" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="C63" s="22"/>
+      <c r="C63" s="13" t="s">
+        <v>68</v>
+      </c>
       <c r="D63" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>